<commit_message>
Added early new unit placement
</commit_message>
<xml_diff>
--- a/Abilities.xlsx
+++ b/Abilities.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9303"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="88">
   <si>
     <t>Name</t>
   </si>
@@ -198,9 +198,6 @@
     <t>Slimey</t>
   </si>
   <si>
-    <t>After dying, deals 3 (Fire) damage to ALL units within 1 cell</t>
-  </si>
-  <si>
     <t>Putrid</t>
   </si>
   <si>
@@ -268,6 +265,21 @@
   </si>
   <si>
     <t>When deploying normally, can only be deployed in the further parts of the deployment zone</t>
+  </si>
+  <si>
+    <t>After dying, deals 2 (Fire) damage to ALL units within 1 cell</t>
+  </si>
+  <si>
+    <t>Woundable</t>
+  </si>
+  <si>
+    <t>If current half is half the maximu or lower, unit gains Weak</t>
+  </si>
+  <si>
+    <t>Unscoring</t>
+  </si>
+  <si>
+    <t>Cannot capture or contest objectives</t>
   </si>
 </sst>
 </file>
@@ -371,7 +383,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -388,13 +400,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="4" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -702,33 +717,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J58"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J62"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.140625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" style="3"/>
-    <col min="3" max="3" width="16.28515625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="72.85546875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="3.85546875" style="3" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="16.109375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" style="3"/>
+    <col min="3" max="3" width="16.33203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="72.88671875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="3.88671875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="17.33203125" style="3" customWidth="1"/>
     <col min="7" max="7" width="45" style="3" customWidth="1"/>
-    <col min="8" max="8" width="12.42578125" style="3" customWidth="1"/>
-    <col min="9" max="9" width="13.42578125" style="3" customWidth="1"/>
-    <col min="10" max="10" width="44.85546875" style="3" customWidth="1"/>
-    <col min="11" max="16384" width="8.85546875" style="3"/>
+    <col min="8" max="8" width="12.44140625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="13.44140625" style="3" customWidth="1"/>
+    <col min="10" max="10" width="44.88671875" style="3" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="14.45" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-    </row>
-    <row r="2" spans="1:10" ht="14.45" x14ac:dyDescent="0.3">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="5"/>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -736,7 +751,7 @@
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -756,10 +771,10 @@
         <v>0</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="14.45" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -783,8 +798,8 @@
       </c>
     </row>
     <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>79</v>
+      <c r="A6" s="6" t="s">
+        <v>78</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>6</v>
@@ -805,22 +820,22 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C8" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F8" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="G8" s="8" t="s">
+      <c r="F8" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="9" t="s">
         <v>25</v>
       </c>
       <c r="I8" s="2" t="s">
@@ -830,17 +845,17 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C9" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="G9" s="8" t="s">
+      <c r="F9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I9" s="2" t="s">
@@ -850,17 +865,17 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C10" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F10" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="G10" s="8" t="s">
+      <c r="F10" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="G10" s="9" t="s">
         <v>26</v>
       </c>
       <c r="I10" s="2" t="s">
@@ -870,17 +885,17 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C12" s="2" t="s">
         <v>0</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F12" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G12" s="4" t="s">
+      <c r="F12" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="G12" s="7" t="s">
         <v>28</v>
       </c>
       <c r="I12" s="2" t="s">
@@ -890,17 +905,17 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C13" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F13" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G13" s="4" t="s">
+      <c r="F13" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G13" s="7" t="s">
         <v>8</v>
       </c>
       <c r="I13" s="2" t="s">
@@ -910,17 +925,17 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="28.9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C14" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G14" s="4" t="s">
+      <c r="F14" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G14" s="7" t="s">
         <v>29</v>
       </c>
       <c r="I14" s="2" t="s">
@@ -930,7 +945,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C16" s="2" t="s">
         <v>0</v>
       </c>
@@ -950,7 +965,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="3:10" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C17" s="2" t="s">
         <v>5</v>
       </c>
@@ -990,7 +1005,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="3:10" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C20" s="2" t="s">
         <v>0</v>
       </c>
@@ -1010,7 +1025,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="3:10" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C21" s="2" t="s">
         <v>5</v>
       </c>
@@ -1030,7 +1045,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="3:10" ht="28.9" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:10" ht="28.95" x14ac:dyDescent="0.3">
       <c r="C22" s="2" t="s">
         <v>6</v>
       </c>
@@ -1050,11 +1065,11 @@
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C24" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="D24" s="8" t="s">
+    <row r="24" spans="3:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="C24" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>24</v>
       </c>
       <c r="F24" s="4" t="s">
@@ -1063,18 +1078,18 @@
       <c r="G24" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="I24" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="J24" s="8" t="s">
+      <c r="I24" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="J24" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C25" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D25" s="8" t="s">
+    <row r="25" spans="3:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="C25" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F25" s="4" t="s">
@@ -1083,18 +1098,18 @@
       <c r="G25" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="I25" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J25" s="8" t="s">
+      <c r="I25" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J25" s="7" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="26" spans="3:10" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C26" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26" s="8" t="s">
+      <c r="C26" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" s="7" t="s">
         <v>27</v>
       </c>
       <c r="F26" s="4" t="s">
@@ -1103,85 +1118,85 @@
       <c r="G26" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="I26" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="J26" s="8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="28" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C28" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D28" s="4" t="s">
+      <c r="I26" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="28" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C28" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G28" s="4" t="s">
+      <c r="F28" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="G28" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="I28" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="J28" s="8" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="29" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C29" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D29" s="4" t="s">
+      <c r="I28" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="J28" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="29" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C29" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F29" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G29" s="4" t="s">
+      <c r="F29" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="G29" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="I29" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J29" s="8" t="s">
+      <c r="I29" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J29" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="3:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="C30" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30" s="4" t="s">
+    <row r="30" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C30" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="F30" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G30" s="4" t="s">
+      <c r="F30" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="G30" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="I30" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="J30" s="8" t="s">
+      <c r="I30" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="J30" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="32" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C32" s="4" t="s">
         <v>0</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F32" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G32" s="4" t="s">
-        <v>78</v>
+      <c r="F32" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>77</v>
       </c>
       <c r="I32" s="4" t="s">
         <v>0</v>
@@ -1197,10 +1212,10 @@
       <c r="D33" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F33" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G33" s="4" t="s">
+      <c r="F33" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="G33" s="9" t="s">
         <v>8</v>
       </c>
       <c r="I33" s="4" t="s">
@@ -1210,18 +1225,18 @@
         <v>17</v>
       </c>
     </row>
-    <row r="34" spans="3:10" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:10" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C34" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F34" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G34" s="4" t="s">
-        <v>60</v>
+      <c r="F34" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>83</v>
       </c>
       <c r="I34" s="4" t="s">
         <v>6</v>
@@ -1230,7 +1245,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="36" spans="3:10" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C36" s="4" t="s">
         <v>0</v>
       </c>
@@ -1241,7 +1256,7 @@
         <v>0</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I36" s="4" t="s">
         <v>0</v>
@@ -1250,7 +1265,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="37" spans="3:10" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="37" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C37" s="4" t="s">
         <v>5</v>
       </c>
@@ -1270,7 +1285,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="38" spans="3:10" ht="28.9" x14ac:dyDescent="0.3">
+    <row r="38" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C38" s="4" t="s">
         <v>6</v>
       </c>
@@ -1281,40 +1296,40 @@
         <v>6</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I38" s="4" t="s">
         <v>6</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="40" spans="3:10" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C40" s="4" t="s">
         <v>0</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="F40"/>
-      <c r="G40"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
       <c r="I40" s="4" t="s">
         <v>0</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="41" spans="3:10" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="41" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C41" s="4" t="s">
         <v>5</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F41"/>
-      <c r="G41"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
       <c r="I41" s="4" t="s">
         <v>5</v>
       </c>
@@ -1322,23 +1337,23 @@
         <v>17</v>
       </c>
     </row>
-    <row r="42" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C42" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="F42"/>
-      <c r="G42"/>
+        <v>66</v>
+      </c>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
       <c r="I42" s="4" t="s">
         <v>6</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="44" spans="3:10" ht="14.45" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="44" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C44" s="4" t="s">
         <v>0</v>
       </c>
@@ -1349,10 +1364,10 @@
         <v>0</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="45" spans="3:10" ht="14.45" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="45" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C45" s="4" t="s">
         <v>5</v>
       </c>
@@ -1366,7 +1381,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="46" spans="3:10" ht="28.9" x14ac:dyDescent="0.3">
+    <row r="46" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C46" s="4" t="s">
         <v>6</v>
       </c>
@@ -1377,24 +1392,24 @@
         <v>6</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="48" spans="3:10" ht="14.45" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="48" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C48" s="4" t="s">
         <v>0</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I48" s="4" t="s">
         <v>0</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="49" spans="3:10" ht="14.45" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="49" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C49" s="4" t="s">
         <v>5</v>
       </c>
@@ -1408,35 +1423,35 @@
         <v>17</v>
       </c>
     </row>
-    <row r="50" spans="3:10" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="50" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C50" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I50" s="4" t="s">
         <v>6</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="52" spans="3:10" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="52" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C52" s="4" t="s">
         <v>0</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I52" s="4" t="s">
         <v>0</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="53" spans="3:10" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="53" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C53" s="4" t="s">
         <v>5</v>
       </c>
@@ -1450,42 +1465,84 @@
         <v>17</v>
       </c>
     </row>
-    <row r="54" spans="3:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="54" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C54" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I54" s="4" t="s">
         <v>6</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="56" spans="3:10" ht="14.45" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="56" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C56" s="4" t="s">
         <v>0</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="57" spans="3:10" ht="14.45" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+      <c r="I56" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J56" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="57" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C57" s="4" t="s">
         <v>5</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="58" spans="3:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I57" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J57" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="58" spans="3:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C58" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
+      </c>
+      <c r="I58" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J58" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="60" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="I60" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J60" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="61" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="I61" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J61" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="62" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="I62" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J62" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -1499,9 +1556,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="12.5703125" customWidth="1"/>
+    <col min="3" max="3" width="12.5546875" customWidth="1"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1511,7 +1568,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed unit deployment bug, item draw bug remains
</commit_message>
<xml_diff>
--- a/Abilities.xlsx
+++ b/Abilities.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="184">
   <si>
     <t>Name</t>
   </si>
@@ -93,9 +93,6 @@
     <t>Covers the cell under unit in "Oil"</t>
   </si>
   <si>
-    <t>First instance of incoming damage deals 0 damage</t>
-  </si>
-  <si>
     <t>Dripping</t>
   </si>
   <si>
@@ -126,9 +123,6 @@
     <t>Infiltrating</t>
   </si>
   <si>
-    <t>Resistant: (Fire/Lightning/Physical)</t>
-  </si>
-  <si>
     <t xml:space="preserve"> -1 (&lt;Damage type&gt;) damage received</t>
   </si>
   <si>
@@ -153,9 +147,6 @@
     <t>Battle-hungry</t>
   </si>
   <si>
-    <t>If hasn't attacked anyone for 2 turns, gains Mad</t>
-  </si>
-  <si>
     <t>Can be deployed in a line right behind enemy's deployment zone, takes 1 extra turn to arrive this way</t>
   </si>
   <si>
@@ -201,24 +192,15 @@
     <t>Applies "Weak" to ALL units within 1 cell</t>
   </si>
   <si>
-    <t>When deployed, places 1 "Stout" and 2 "Sparrow" units</t>
-  </si>
-  <si>
     <t>Bloodthirsty</t>
   </si>
   <si>
-    <t>Can also attack friendly units</t>
-  </si>
-  <si>
     <t>Vampiric</t>
   </si>
   <si>
     <t>Decaying</t>
   </si>
   <si>
-    <t>After beign moved, takes 1 (Physical) damage</t>
-  </si>
-  <si>
     <t>A game of skeletons</t>
   </si>
   <si>
@@ -237,9 +219,6 @@
     <t>At the start of each turn, has 50% chance to gain either "Beckoned" or "Cowardly"</t>
   </si>
   <si>
-    <t>Vulnerable:(Fire/Lightning/Physical)</t>
-  </si>
-  <si>
     <t>Delayed</t>
   </si>
   <si>
@@ -249,9 +228,6 @@
     <t>Woundable</t>
   </si>
   <si>
-    <t>If current half is half the maximu or lower, unit gains Weak</t>
-  </si>
-  <si>
     <t>Unscoring</t>
   </si>
   <si>
@@ -444,9 +420,6 @@
     <t>Name: Base names alphabetically arranged, then abilities additions</t>
   </si>
   <si>
-    <t>At the start of the round, creates a 'Skelic' unit nearby. Afterwards, if if this unit is standing next to 2 or more units with this Ability, it is immedeatly destroyed</t>
-  </si>
-  <si>
     <t>At the start of the round, Merges with all units within 1 cell with this ability</t>
   </si>
   <si>
@@ -483,12 +456,6 @@
     <t>Deals 1 (Physical) damage to all enemies within a 2 cell square ring</t>
   </si>
   <si>
-    <t>""</t>
-  </si>
-  <si>
-    <t>Functions as temporary additional maximum health, but is only restored when additional "Extra health (X)" ability is applied</t>
-  </si>
-  <si>
     <t>Extra healthy (X)</t>
   </si>
   <si>
@@ -499,6 +466,108 @@
   </si>
   <si>
     <t>The first time player uses an item when this unit is on the battlefield, another item is immedeatly drawn</t>
+  </si>
+  <si>
+    <t>After being moved, takes 1 (Physical) damage</t>
+  </si>
+  <si>
+    <t>If hasn't attacked anyone for 2 turns, gains Beckoned</t>
+  </si>
+  <si>
+    <t>Vulnerable:(&lt;Damage type&gt;)</t>
+  </si>
+  <si>
+    <t>Resistant: (&lt;Damage type&gt;)</t>
+  </si>
+  <si>
+    <t>explosive ""</t>
+  </si>
+  <si>
+    <t>sneaky ""</t>
+  </si>
+  <si>
+    <t>When deployed, places 1 "Stout" and 2 "Sparrow" units what gain other abilities of the unit</t>
+  </si>
+  <si>
+    <t>adaptive ""</t>
+  </si>
+  <si>
+    <t>Adaptive (&lt;Damage type&gt;)</t>
+  </si>
+  <si>
+    <t>After taking damage, gains resistance to the type of damage dealt</t>
+  </si>
+  <si>
+    <t>Slowed</t>
+  </si>
+  <si>
+    <t>After moving, must remain stationary next turn</t>
+  </si>
+  <si>
+    <t>Paranoid</t>
+  </si>
+  <si>
+    <t>If deployed closer than 3 cells away from any other units, until the end of the battle, maximum health is decreased by 3 (To a minimum of 1)</t>
+  </si>
+  <si>
+    <t>Terrified</t>
+  </si>
+  <si>
+    <t>At the end of the turn, if no other friendly units are within 3 cells of this unit, this unit takes 1 (Mental) damage</t>
+  </si>
+  <si>
+    <t>Damage types:</t>
+  </si>
+  <si>
+    <t>Physical</t>
+  </si>
+  <si>
+    <t>Lightning</t>
+  </si>
+  <si>
+    <t>Fire</t>
+  </si>
+  <si>
+    <t>Frost</t>
+  </si>
+  <si>
+    <t>Poison</t>
+  </si>
+  <si>
+    <t>Mental</t>
+  </si>
+  <si>
+    <t>Costly</t>
+  </si>
+  <si>
+    <t>While this unit is a part of your army, you lose 1$ at the end of each shop</t>
+  </si>
+  <si>
+    <t>If current half is half the maximum or lower, unit gains Weak</t>
+  </si>
+  <si>
+    <t>battle hungry ()</t>
+  </si>
+  <si>
+    <t>Attacks also target and damage friendly units</t>
+  </si>
+  <si>
+    <t>"" watched at by Gods</t>
+  </si>
+  <si>
+    <t>Watched by Gods</t>
+  </si>
+  <si>
+    <t>Each time a unit within 1 cells is destroyed, until the end of the Battle, this unit gains a random Ability</t>
+  </si>
+  <si>
+    <t>Has (X) amount of additional maximum health which cannot be healed</t>
+  </si>
+  <si>
+    <t>At the start of the round, creates a 'Skelic' unit nearby. Afterwards, if this unit is standing next to 2 or more units, it is immedeatly destroyed</t>
+  </si>
+  <si>
+    <t>Next instance of incoming damage deals 0 damage. Functions once per battle</t>
   </si>
 </sst>
 </file>
@@ -579,7 +648,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -639,6 +708,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -647,7 +731,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -681,6 +765,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1000,7 +1090,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J106"/>
+  <dimension ref="A1:J112"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.109375" style="3" customWidth="1"/>
@@ -1017,18 +1107,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="5"/>
@@ -1038,7 +1128,7 @@
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
     </row>
-    <row r="4" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1046,7 +1136,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>36</v>
+        <v>153</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>0</v>
@@ -1058,28 +1148,28 @@
         <v>0</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>73</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="C5" s="1" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -1107,13 +1197,13 @@
     </row>
     <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>6</v>
@@ -1125,7 +1215,7 @@
         <v>6</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
@@ -1133,12 +1223,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C9" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>0</v>
@@ -1153,27 +1243,33 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="14" t="s">
+        <v>166</v>
+      </c>
       <c r="C10" s="1" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>167</v>
+      </c>
       <c r="C11" s="1" t="s">
         <v>5</v>
       </c>
@@ -1194,11 +1290,14 @@
       </c>
     </row>
     <row r="12" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>168</v>
+      </c>
       <c r="C12" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>6</v>
@@ -1213,7 +1312,15 @@
         <v>18</v>
       </c>
     </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>170</v>
+      </c>
       <c r="C14" s="2" t="s">
         <v>0</v>
       </c>
@@ -1224,36 +1331,42 @@
         <v>0</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I14" s="4" t="s">
         <v>0</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>171</v>
+      </c>
       <c r="C15" s="2" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>172</v>
+      </c>
       <c r="C16" s="2" t="s">
         <v>5</v>
       </c>
@@ -1284,13 +1397,13 @@
         <v>6</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>6</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
     </row>
     <row r="19" spans="3:10" x14ac:dyDescent="0.3">
@@ -1304,7 +1417,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>0</v>
@@ -1335,22 +1448,22 @@
     </row>
     <row r="21" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="C21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="J21" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="22" spans="3:10" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1364,7 +1477,7 @@
         <v>6</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>6</v>
@@ -1378,39 +1491,39 @@
         <v>0</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>0</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I24" s="4" t="s">
         <v>0</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="C25" s="2" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="3:10" x14ac:dyDescent="0.3">
@@ -1438,19 +1551,19 @@
         <v>6</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="I27" s="4" t="s">
         <v>6</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="29" spans="3:10" x14ac:dyDescent="0.3">
@@ -1464,7 +1577,7 @@
         <v>0</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I29" s="7" t="s">
         <v>0</v>
@@ -1475,22 +1588,22 @@
     </row>
     <row r="30" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="C30" s="7" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
     </row>
     <row r="31" spans="3:10" x14ac:dyDescent="0.3">
@@ -1513,24 +1626,24 @@
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="3:10" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:10" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C32" s="7" t="s">
         <v>6</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>25</v>
+        <v>183</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I32" s="7" t="s">
         <v>6</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="34" spans="3:10" x14ac:dyDescent="0.3">
@@ -1538,39 +1651,39 @@
         <v>0</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F34" s="8" t="s">
         <v>0</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="I34" s="7" t="s">
         <v>0</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="35" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="C35" s="7" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="I35" s="7" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="J35" s="7" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="36" spans="3:10" x14ac:dyDescent="0.3">
@@ -1598,19 +1711,19 @@
         <v>6</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F37" s="8" t="s">
         <v>6</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I37" s="7" t="s">
         <v>6</v>
       </c>
       <c r="J37" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="3:10" x14ac:dyDescent="0.3">
@@ -1618,965 +1731,1137 @@
         <v>0</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F39" s="8" t="s">
         <v>0</v>
       </c>
       <c r="G39" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J39" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="40" spans="3:10" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C40" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="G40" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="J40" s="4" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="41" spans="3:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C41" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G41" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J41" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="42" spans="3:10" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C42" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G42" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="I42" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J42" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="44" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C44" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="I44" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J44" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="45" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C45" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="I45" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="J45" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="46" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C46" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I46" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J46" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="47" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C47" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="I47" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J47" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="49" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C49" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I49" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J49" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="50" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C50" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="I50" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="J50" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="51" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C51" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I51" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J51" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="52" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C52" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="I52" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J52" s="4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="53" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="F53" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="G53" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="54" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C54" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F54" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="G54" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="I54" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J54" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="55" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C55" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F55" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="G55" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="I55" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="J55" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="56" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C56" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I56" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J56" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="57" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C57" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="I57" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J57" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="59" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C59" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="I59" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J59" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="60" spans="3:10" s="10" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C60" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="G60" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="I60" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="J60" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="61" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C61" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G61" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I61" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J61" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="62" spans="3:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C62" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F62" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I62" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J62" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="64" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C64" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F64" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G64" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="I64" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J64" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="65" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C65" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="G65" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="I65" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="J65" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="66" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C66" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F66" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G66" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I66" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J66" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="67" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C67" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G67" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="I67" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J67" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="69" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C69" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G69" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I69" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J69" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="70" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C70" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F70" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="G70" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="I70" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="J70" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="71" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C71" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D71" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G71" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I71" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J71" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="72" spans="3:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C72" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G72" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="I72" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J72" s="4" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="74" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C74" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="F74" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G74" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="I74" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J74" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="I39" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="J39" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="40" spans="3:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C40" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D40" s="4" t="s">
+    </row>
+    <row r="75" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C75" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="G75" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="I75" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="J75" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="76" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C76" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D76" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F40" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="G40" s="8" t="s">
+      <c r="F76" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G76" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="I40" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="J40" s="4" t="s">
+      <c r="I76" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J76" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="41" spans="3:10" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C41" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="F41" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="G41" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="I41" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="J41" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="43" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C43" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="F43" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G43" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="I43" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="J43" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="44" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C44" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="F44" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="G44" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="I44" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="J44" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="45" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C45" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F45" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G45" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="I45" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="J45" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="46" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C46" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="F46" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G46" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="I46" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="J46" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="48" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C48" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="F48" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="I48" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="J48" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="49" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C49" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="F49" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="G49" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="I49" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="J49" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="50" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C50" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F50" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G50" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="I50" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="J50" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="51" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C51" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="F51" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G51" s="4" t="s">
+    <row r="77" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C77" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G77" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="I77" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J77" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="79" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C79" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D79" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="I51" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="J51" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="52" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="F52" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="G52" s="9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="53" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C53" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F53" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="G53" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="I53" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="J53" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="54" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C54" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="D54" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="F54" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="G54" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="I54" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="J54" s="4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="55" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C55" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="I55" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="J55" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="56" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C56" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D56" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="I56" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="J56" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="58" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C58" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D58" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="F58" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G58" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="I58" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="J58" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="59" spans="3:10" s="10" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C59" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="D59" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="F59" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="G59" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="I59" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="J59" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="60" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C60" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D60" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F60" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G60" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="I60" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="J60" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="61" spans="3:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="C61" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D61" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F61" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G61" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="I61" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="J61" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="63" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C63" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D63" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="F63" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G63" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="I63" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="J63" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="64" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C64" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="D64" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="F64" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="G64" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="I64" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="J64" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="65" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C65" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D65" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F65" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G65" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="I65" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="J65" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="66" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C66" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D66" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="F66" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G66" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="I66" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="J66" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="68" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C68" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D68" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="F68" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G68" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="I68" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="J68" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="69" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C69" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="D69" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="F69" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="G69" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="I69" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="J69" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="70" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C70" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D70" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F70" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G70" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="I70" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="J70" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="71" spans="3:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C71" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D71" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="F71" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G71" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="I71" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="J71" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="73" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C73" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D73" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="F73" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G73" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="I73" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="J73" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="74" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C74" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="D74" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="F74" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="G74" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="I74" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="J74" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="75" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C75" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D75" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F75" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G75" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="I75" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="J75" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="76" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C76" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D76" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="F76" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G76" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="I76" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="J76" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="78" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C78" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D78" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="F78" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G78" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="I78" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="J78" s="4" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="79" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C79" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="D79" s="4" t="s">
-        <v>104</v>
-      </c>
       <c r="F79" s="4" t="s">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>103</v>
+        <v>0</v>
       </c>
       <c r="J79" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="80" spans="3:10" x14ac:dyDescent="0.3">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="80" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="C80" s="4" t="s">
-        <v>5</v>
+        <v>112</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>12</v>
+        <v>96</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>5</v>
+        <v>112</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>8</v>
+        <v>96</v>
       </c>
       <c r="I80" s="4" t="s">
-        <v>5</v>
+        <v>95</v>
       </c>
       <c r="J80" s="4" t="s">
-        <v>17</v>
+        <v>96</v>
       </c>
     </row>
     <row r="81" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C81" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>91</v>
+        <v>12</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J81" s="4" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="83" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C83" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D83" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="F83" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G83" s="4" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="84" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="82" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C82" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F82" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G82" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="I82" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J82" s="4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="84" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C84" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F84" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G84" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="I84" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J84" s="4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="85" spans="3:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C85" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="G85" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="I85" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="J85" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="86" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C86" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D86" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F86" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G86" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I86" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J86" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="87" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C87" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="F87" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G87" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="I87" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J87" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="88" spans="3:10" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F88" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="G88" s="9" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="89" spans="3:10" ht="24" x14ac:dyDescent="0.3">
+      <c r="C89" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="F89" s="17"/>
+      <c r="G89" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="D84" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="F84" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="G84" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="85" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C85" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D85" s="4" t="s">
+    </row>
+    <row r="90" spans="3:10" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C90" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D90" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="F90" s="17"/>
+      <c r="G90" s="9" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="91" spans="3:10" ht="24" x14ac:dyDescent="0.3">
+      <c r="C91" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D91" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F85" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G85" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="86" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C86" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D86" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="F86" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G86" s="4" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="87" spans="3:10" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F87" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G87" s="9" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="88" spans="3:10" ht="24" x14ac:dyDescent="0.3">
-      <c r="C88" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D88" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="F88" s="15"/>
-      <c r="G88" s="9" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="89" spans="3:10" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C89" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="D89" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="F89" s="15"/>
-      <c r="G89" s="9" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="90" spans="3:10" ht="24" x14ac:dyDescent="0.3">
-      <c r="C90" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D90" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F90" s="16"/>
-      <c r="G90" s="9" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="91" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C91" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D91" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="F91" s="11"/>
-      <c r="G91"/>
+      <c r="F91" s="18"/>
+      <c r="G91" s="9" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="92" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C92" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D92" s="4" t="s">
+        <v>145</v>
+      </c>
       <c r="F92" s="11"/>
       <c r="G92"/>
     </row>
     <row r="93" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C93" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D93" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F93" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G93" s="4" t="s">
-        <v>129</v>
-      </c>
+      <c r="F93" s="11"/>
+      <c r="G93"/>
     </row>
     <row r="94" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C94" s="4" t="s">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>104</v>
+        <v>121</v>
+      </c>
+      <c r="I94" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J94" s="4" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="95" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C95" s="4" t="s">
-        <v>5</v>
+        <v>112</v>
       </c>
       <c r="D95" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="I95" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="J95" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="96" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C96" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D96" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F95" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G95" s="4" t="s">
+      <c r="F96" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G96" s="4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="96" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C96" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D96" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="F96" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G96" s="4" t="s">
+      <c r="I96" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J96" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="97" spans="3:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C97" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G97" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="I97" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J97" s="4" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="98" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C98"/>
+      <c r="D98"/>
+      <c r="F98" s="12"/>
+      <c r="G98" s="12"/>
+    </row>
+    <row r="99" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C99" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D99" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F99" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G99" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="I99" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J99" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="100" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C100" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F100" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="G100" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="I100" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="J100" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="101" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C101" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G101" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I101" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J101" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="102" spans="3:10" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C102" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="F102" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G102" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="I102" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J102" s="4" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="104" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C104" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D104" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="F104" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G104" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="I104" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J104" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="105" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C105" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="F105" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="G105" s="4" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="97" spans="3:7" x14ac:dyDescent="0.3">
-      <c r="C97"/>
-      <c r="D97"/>
-      <c r="F97" s="12"/>
-      <c r="G97" s="12"/>
-    </row>
-    <row r="98" spans="3:7" x14ac:dyDescent="0.3">
-      <c r="C98" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D98" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="F98" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G98" s="4" t="s">
+      <c r="I105" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="J105" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="106" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C106" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D106" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F106" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G106" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I106" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J106" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="107" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C107" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G107" s="4" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="99" spans="3:7" x14ac:dyDescent="0.3">
-      <c r="C99" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="D99" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="F99" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="G99" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="100" spans="3:7" x14ac:dyDescent="0.3">
-      <c r="C100" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D100" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F100" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G100" s="4" t="s">
+      <c r="I107" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J107" s="4" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="109" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="F109" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G109" s="4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="110" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="F110" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="G110" s="4" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="111" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="F111" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G111" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="101" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C101" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D101" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="F101" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G101" s="4" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="103" spans="3:7" x14ac:dyDescent="0.3">
-      <c r="F103" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G103" s="4" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="104" spans="3:7" x14ac:dyDescent="0.3">
-      <c r="F104" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="G104" s="4" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="105" spans="3:7" x14ac:dyDescent="0.3">
-      <c r="F105" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G105" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="106" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="F106" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G106" s="4" t="s">
-        <v>139</v>
+    <row r="112" spans="3:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F112" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G112" s="4" t="s">
+        <v>180</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="F87:F90"/>
+    <mergeCell ref="F88:F91"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>